<commit_message>
Cập nhật nội dung README
</commit_message>
<xml_diff>
--- a/abc_analyst.xlsx
+++ b/abc_analyst.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\OneDrive\Máy tính\VTI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EBCBC8D-8068-4383-9777-25A5B2DAACBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9EE5632-AAD3-4D0A-A117-9145D452C073}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{72632174-C81A-43E7-BC36-DD75E61563EA}"/>
+    <workbookView xWindow="1920" yWindow="1920" windowWidth="16764" windowHeight="8964" activeTab="1" xr2:uid="{72632174-C81A-43E7-BC36-DD75E61563EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Pivot" sheetId="2" r:id="rId1"/>
@@ -23,7 +23,7 @@
   </externalReferences>
   <calcPr calcId="181029"/>
   <pivotCaches>
-    <pivotCache cacheId="24" r:id="rId6"/>
+    <pivotCache cacheId="0" r:id="rId6"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -3631,12 +3631,12 @@
       <sheetName val="⚠️ Cần Review"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
       <sheetData sheetId="6">
         <row r="1">
           <cell r="A1" t="str">
@@ -8279,10 +8279,10 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
+      <sheetData sheetId="7" refreshError="1"/>
+      <sheetData sheetId="8" refreshError="1"/>
+      <sheetData sheetId="9" refreshError="1"/>
+      <sheetData sheetId="10" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -23613,7 +23613,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EE97F5BA-A452-45B6-BCCF-ACA9B28456C3}" name="PivotTable1" cacheId="24" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EE97F5BA-A452-45B6-BCCF-ACA9B28456C3}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A3:E224" firstHeaderRow="0" firstDataRow="1" firstDataCol="2"/>
   <pivotFields count="19">
     <pivotField compact="0" outline="0" showAll="0">

</xml_diff>